<commit_message>
minor corrections in unit conversion factors (mainly operation of SUVs)
</commit_message>
<xml_diff>
--- a/docs/_static/unit_conversion_energyscope.xlsx
+++ b/docs/_static/unit_conversion_energyscope.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="5605" uniqueCount="1364">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="5599" uniqueCount="1363">
   <si>
     <t>Name</t>
   </si>
@@ -3936,9 +3936,6 @@
   </si>
   <si>
     <t>payload (6.3 t): (Sacchi, 2021)</t>
-  </si>
-  <si>
-    <t>natural gas LHV (13.1 kWh/kg), natural gas density (0.777 kg/m3): (Engineering ToolBox, 2003)</t>
   </si>
   <si>
     <t>electricity consumption (42.3 kWh/kg H2): (Gerloff, 2021), LHV hydrogen (33.3 kWh/kg): (Engineering ToolBox, 2003), capacity (1 MWe)</t>
@@ -4464,7 +4461,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:G934"/>
+  <dimension ref="A1:G933"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:7">
@@ -14464,7 +14461,7 @@
         <v>0</v>
       </c>
       <c r="E420" t="s">
-        <v>1124</v>
+        <v>1121</v>
       </c>
       <c r="F420" t="s">
         <v>1123</v>
@@ -14704,7 +14701,7 @@
         <v>0</v>
       </c>
       <c r="E430" t="s">
-        <v>1124</v>
+        <v>1121</v>
       </c>
       <c r="F430" t="s">
         <v>1123</v>
@@ -14724,7 +14721,7 @@
         <v>839</v>
       </c>
       <c r="D431">
-        <f>1 / (0.777 * 13.1)</f>
+        <f>1 * 3.6 / 39</f>
         <v>0</v>
       </c>
       <c r="E431" t="s">
@@ -14748,7 +14745,7 @@
         <v>839</v>
       </c>
       <c r="D432">
-        <f>1 / (0.777 * 13.1)</f>
+        <f>1 * 3.6 / 39</f>
         <v>0</v>
       </c>
       <c r="E432" t="s">
@@ -17585,7 +17582,7 @@
         <v>914</v>
       </c>
       <c r="D551">
-        <f>1 / (0.777 * 13.1)</f>
+        <f> 3.6 / 39</f>
         <v>0</v>
       </c>
       <c r="E551" t="s">
@@ -17595,7 +17592,7 @@
         <v>1123</v>
       </c>
       <c r="G551" t="s">
-        <v>1307</v>
+        <v>1274</v>
       </c>
     </row>
     <row r="552" spans="1:7">
@@ -17609,7 +17606,7 @@
         <v>915</v>
       </c>
       <c r="D552">
-        <f>1 / (0.777 * 13.1)</f>
+        <f> 3.6 / 39</f>
         <v>0</v>
       </c>
       <c r="E552" t="s">
@@ -17619,7 +17616,7 @@
         <v>1123</v>
       </c>
       <c r="G552" t="s">
-        <v>1307</v>
+        <v>1274</v>
       </c>
     </row>
     <row r="553" spans="1:7">
@@ -17643,7 +17640,7 @@
         <v>1125</v>
       </c>
       <c r="G553" t="s">
-        <v>1308</v>
+        <v>1307</v>
       </c>
     </row>
     <row r="554" spans="1:7">
@@ -17830,7 +17827,7 @@
         <v>1131</v>
       </c>
       <c r="G561" t="s">
-        <v>1309</v>
+        <v>1308</v>
       </c>
     </row>
     <row r="562" spans="1:7">
@@ -17877,7 +17874,7 @@
         <v>1131</v>
       </c>
       <c r="G563" t="s">
-        <v>1309</v>
+        <v>1308</v>
       </c>
     </row>
     <row r="564" spans="1:7">
@@ -17924,7 +17921,7 @@
         <v>1131</v>
       </c>
       <c r="G565" t="s">
-        <v>1309</v>
+        <v>1308</v>
       </c>
     </row>
     <row r="566" spans="1:7">
@@ -18056,17 +18053,17 @@
         <v>927</v>
       </c>
       <c r="D571">
-        <f>1</f>
+        <f>1/1.23</f>
         <v>0</v>
       </c>
       <c r="E571" t="s">
-        <v>1126</v>
+        <v>1127</v>
       </c>
       <c r="F571" t="s">
         <v>1126</v>
       </c>
       <c r="G571" t="s">
-        <v>1137</v>
+        <v>1158</v>
       </c>
     </row>
     <row r="572" spans="1:7">
@@ -18104,17 +18101,17 @@
         <v>928</v>
       </c>
       <c r="D573">
-        <f>1</f>
+        <f>1/1.23</f>
         <v>0</v>
       </c>
       <c r="E573" t="s">
-        <v>1126</v>
+        <v>1127</v>
       </c>
       <c r="F573" t="s">
         <v>1126</v>
       </c>
       <c r="G573" t="s">
-        <v>1137</v>
+        <v>1158</v>
       </c>
     </row>
     <row r="574" spans="1:7">
@@ -18152,17 +18149,17 @@
         <v>929</v>
       </c>
       <c r="D575">
-        <f>1</f>
+        <f>1/1.23</f>
         <v>0</v>
       </c>
       <c r="E575" t="s">
-        <v>1126</v>
+        <v>1127</v>
       </c>
       <c r="F575" t="s">
         <v>1126</v>
       </c>
       <c r="G575" t="s">
-        <v>1137</v>
+        <v>1158</v>
       </c>
     </row>
     <row r="576" spans="1:7">
@@ -18200,17 +18197,17 @@
         <v>930</v>
       </c>
       <c r="D577">
-        <f>1</f>
+        <f>1/1.23</f>
         <v>0</v>
       </c>
       <c r="E577" t="s">
-        <v>1126</v>
+        <v>1127</v>
       </c>
       <c r="F577" t="s">
         <v>1126</v>
       </c>
       <c r="G577" t="s">
-        <v>1137</v>
+        <v>1158</v>
       </c>
     </row>
     <row r="578" spans="1:7">
@@ -18248,17 +18245,17 @@
         <v>931</v>
       </c>
       <c r="D579">
-        <f>1</f>
+        <f>1/1.23</f>
         <v>0</v>
       </c>
       <c r="E579" t="s">
-        <v>1126</v>
+        <v>1127</v>
       </c>
       <c r="F579" t="s">
         <v>1126</v>
       </c>
       <c r="G579" t="s">
-        <v>1137</v>
+        <v>1158</v>
       </c>
     </row>
     <row r="580" spans="1:7">
@@ -18296,17 +18293,17 @@
         <v>932</v>
       </c>
       <c r="D581">
-        <f>1</f>
+        <f>1/1.23</f>
         <v>0</v>
       </c>
       <c r="E581" t="s">
-        <v>1126</v>
+        <v>1127</v>
       </c>
       <c r="F581" t="s">
         <v>1126</v>
       </c>
       <c r="G581" t="s">
-        <v>1137</v>
+        <v>1158</v>
       </c>
     </row>
     <row r="582" spans="1:7">
@@ -18344,17 +18341,17 @@
         <v>933</v>
       </c>
       <c r="D583">
-        <f>1</f>
+        <f>1/1.23</f>
         <v>0</v>
       </c>
       <c r="E583" t="s">
-        <v>1126</v>
+        <v>1127</v>
       </c>
       <c r="F583" t="s">
         <v>1126</v>
       </c>
       <c r="G583" t="s">
-        <v>1137</v>
+        <v>1158</v>
       </c>
     </row>
     <row r="584" spans="1:7">
@@ -18392,17 +18389,17 @@
         <v>934</v>
       </c>
       <c r="D585">
-        <f>1</f>
+        <f>1/1.23</f>
         <v>0</v>
       </c>
       <c r="E585" t="s">
-        <v>1126</v>
+        <v>1127</v>
       </c>
       <c r="F585" t="s">
         <v>1126</v>
       </c>
       <c r="G585" t="s">
-        <v>1137</v>
+        <v>1158</v>
       </c>
     </row>
     <row r="586" spans="1:7">
@@ -18440,17 +18437,17 @@
         <v>935</v>
       </c>
       <c r="D587">
-        <f>1</f>
+        <f>1/1.23</f>
         <v>0</v>
       </c>
       <c r="E587" t="s">
-        <v>1126</v>
+        <v>1127</v>
       </c>
       <c r="F587" t="s">
         <v>1126</v>
       </c>
       <c r="G587" t="s">
-        <v>1137</v>
+        <v>1158</v>
       </c>
     </row>
     <row r="588" spans="1:7">
@@ -18488,17 +18485,17 @@
         <v>936</v>
       </c>
       <c r="D589">
-        <f>1</f>
+        <f>1/1.23</f>
         <v>0</v>
       </c>
       <c r="E589" t="s">
-        <v>1126</v>
+        <v>1127</v>
       </c>
       <c r="F589" t="s">
         <v>1126</v>
       </c>
       <c r="G589" t="s">
-        <v>1137</v>
+        <v>1158</v>
       </c>
     </row>
     <row r="590" spans="1:7">
@@ -18536,17 +18533,17 @@
         <v>937</v>
       </c>
       <c r="D591">
-        <f>1</f>
+        <f>1/1.23</f>
         <v>0</v>
       </c>
       <c r="E591" t="s">
-        <v>1126</v>
+        <v>1127</v>
       </c>
       <c r="F591" t="s">
         <v>1126</v>
       </c>
       <c r="G591" t="s">
-        <v>1137</v>
+        <v>1158</v>
       </c>
     </row>
     <row r="592" spans="1:7">
@@ -18584,17 +18581,17 @@
         <v>938</v>
       </c>
       <c r="D593">
-        <f>1</f>
+        <f>1/1.23</f>
         <v>0</v>
       </c>
       <c r="E593" t="s">
-        <v>1126</v>
+        <v>1127</v>
       </c>
       <c r="F593" t="s">
         <v>1126</v>
       </c>
       <c r="G593" t="s">
-        <v>1137</v>
+        <v>1158</v>
       </c>
     </row>
     <row r="594" spans="1:7">
@@ -18618,7 +18615,7 @@
         <v>1125</v>
       </c>
       <c r="G594" t="s">
-        <v>1310</v>
+        <v>1309</v>
       </c>
     </row>
     <row r="595" spans="1:7">
@@ -18666,7 +18663,7 @@
         <v>1123</v>
       </c>
       <c r="G596" t="s">
-        <v>1311</v>
+        <v>1310</v>
       </c>
     </row>
     <row r="597" spans="1:7">
@@ -18828,7 +18825,7 @@
         <v>1132</v>
       </c>
       <c r="G603" t="s">
-        <v>1312</v>
+        <v>1311</v>
       </c>
     </row>
     <row r="604" spans="1:7">
@@ -18876,7 +18873,7 @@
         <v>1132</v>
       </c>
       <c r="G605" t="s">
-        <v>1312</v>
+        <v>1311</v>
       </c>
     </row>
     <row r="606" spans="1:7">
@@ -18924,7 +18921,7 @@
         <v>1133</v>
       </c>
       <c r="G607" t="s">
-        <v>1313</v>
+        <v>1312</v>
       </c>
     </row>
     <row r="608" spans="1:7">
@@ -18971,7 +18968,7 @@
         <v>1133</v>
       </c>
       <c r="G609" t="s">
-        <v>1313</v>
+        <v>1312</v>
       </c>
     </row>
     <row r="610" spans="1:7">
@@ -19018,7 +19015,7 @@
         <v>1133</v>
       </c>
       <c r="G611" t="s">
-        <v>1313</v>
+        <v>1312</v>
       </c>
     </row>
     <row r="612" spans="1:7">
@@ -19065,7 +19062,7 @@
         <v>1133</v>
       </c>
       <c r="G613" t="s">
-        <v>1314</v>
+        <v>1313</v>
       </c>
     </row>
     <row r="614" spans="1:7">
@@ -19113,7 +19110,7 @@
         <v>1133</v>
       </c>
       <c r="G615" t="s">
-        <v>1313</v>
+        <v>1312</v>
       </c>
     </row>
     <row r="616" spans="1:7">
@@ -19160,7 +19157,7 @@
         <v>1132</v>
       </c>
       <c r="G617" t="s">
-        <v>1312</v>
+        <v>1311</v>
       </c>
     </row>
     <row r="618" spans="1:7">
@@ -19208,7 +19205,7 @@
         <v>1132</v>
       </c>
       <c r="G619" t="s">
-        <v>1312</v>
+        <v>1311</v>
       </c>
     </row>
     <row r="620" spans="1:7">
@@ -19256,7 +19253,7 @@
         <v>1132</v>
       </c>
       <c r="G621" t="s">
-        <v>1315</v>
+        <v>1314</v>
       </c>
     </row>
     <row r="622" spans="1:7">
@@ -19304,7 +19301,7 @@
         <v>1133</v>
       </c>
       <c r="G623" t="s">
-        <v>1316</v>
+        <v>1315</v>
       </c>
     </row>
     <row r="624" spans="1:7">
@@ -19328,7 +19325,7 @@
         <v>1130</v>
       </c>
       <c r="G624" t="s">
-        <v>1317</v>
+        <v>1316</v>
       </c>
     </row>
     <row r="625" spans="1:7">
@@ -19352,7 +19349,7 @@
         <v>1133</v>
       </c>
       <c r="G625" t="s">
-        <v>1316</v>
+        <v>1315</v>
       </c>
     </row>
     <row r="626" spans="1:7">
@@ -19376,7 +19373,7 @@
         <v>1130</v>
       </c>
       <c r="G626" t="s">
-        <v>1317</v>
+        <v>1316</v>
       </c>
     </row>
     <row r="627" spans="1:7">
@@ -19400,7 +19397,7 @@
         <v>1133</v>
       </c>
       <c r="G627" t="s">
-        <v>1316</v>
+        <v>1315</v>
       </c>
     </row>
     <row r="628" spans="1:7">
@@ -19424,7 +19421,7 @@
         <v>1130</v>
       </c>
       <c r="G628" t="s">
-        <v>1317</v>
+        <v>1316</v>
       </c>
     </row>
     <row r="629" spans="1:7">
@@ -19448,7 +19445,7 @@
         <v>1133</v>
       </c>
       <c r="G629" t="s">
-        <v>1316</v>
+        <v>1315</v>
       </c>
     </row>
     <row r="630" spans="1:7">
@@ -19472,7 +19469,7 @@
         <v>1130</v>
       </c>
       <c r="G630" t="s">
-        <v>1317</v>
+        <v>1316</v>
       </c>
     </row>
     <row r="631" spans="1:7">
@@ -19496,7 +19493,7 @@
         <v>1133</v>
       </c>
       <c r="G631" t="s">
-        <v>1316</v>
+        <v>1315</v>
       </c>
     </row>
     <row r="632" spans="1:7">
@@ -19543,7 +19540,7 @@
         <v>1133</v>
       </c>
       <c r="G633" t="s">
-        <v>1316</v>
+        <v>1315</v>
       </c>
     </row>
     <row r="634" spans="1:7">
@@ -19567,7 +19564,7 @@
         <v>1130</v>
       </c>
       <c r="G634" t="s">
-        <v>1317</v>
+        <v>1316</v>
       </c>
     </row>
     <row r="635" spans="1:7">
@@ -19591,7 +19588,7 @@
         <v>1133</v>
       </c>
       <c r="G635" t="s">
-        <v>1316</v>
+        <v>1315</v>
       </c>
     </row>
     <row r="636" spans="1:7">
@@ -19615,7 +19612,7 @@
         <v>1130</v>
       </c>
       <c r="G636" t="s">
-        <v>1317</v>
+        <v>1316</v>
       </c>
     </row>
     <row r="637" spans="1:7">
@@ -19639,7 +19636,7 @@
         <v>1133</v>
       </c>
       <c r="G637" t="s">
-        <v>1316</v>
+        <v>1315</v>
       </c>
     </row>
     <row r="638" spans="1:7">
@@ -19663,7 +19660,7 @@
         <v>1130</v>
       </c>
       <c r="G638" t="s">
-        <v>1317</v>
+        <v>1316</v>
       </c>
     </row>
     <row r="639" spans="1:7">
@@ -19687,7 +19684,7 @@
         <v>1133</v>
       </c>
       <c r="G639" t="s">
-        <v>1318</v>
+        <v>1317</v>
       </c>
     </row>
     <row r="640" spans="1:7">
@@ -19711,7 +19708,7 @@
         <v>1130</v>
       </c>
       <c r="G640" t="s">
-        <v>1319</v>
+        <v>1318</v>
       </c>
     </row>
     <row r="641" spans="1:7">
@@ -19735,7 +19732,7 @@
         <v>1133</v>
       </c>
       <c r="G641" t="s">
-        <v>1318</v>
+        <v>1317</v>
       </c>
     </row>
     <row r="642" spans="1:7">
@@ -19759,7 +19756,7 @@
         <v>1130</v>
       </c>
       <c r="G642" t="s">
-        <v>1319</v>
+        <v>1318</v>
       </c>
     </row>
     <row r="643" spans="1:7">
@@ -19783,7 +19780,7 @@
         <v>1133</v>
       </c>
       <c r="G643" t="s">
-        <v>1318</v>
+        <v>1317</v>
       </c>
     </row>
     <row r="644" spans="1:7">
@@ -19807,7 +19804,7 @@
         <v>1130</v>
       </c>
       <c r="G644" t="s">
-        <v>1319</v>
+        <v>1318</v>
       </c>
     </row>
     <row r="645" spans="1:7">
@@ -19831,7 +19828,7 @@
         <v>1133</v>
       </c>
       <c r="G645" t="s">
-        <v>1318</v>
+        <v>1317</v>
       </c>
     </row>
     <row r="646" spans="1:7">
@@ -19855,7 +19852,7 @@
         <v>1130</v>
       </c>
       <c r="G646" t="s">
-        <v>1319</v>
+        <v>1318</v>
       </c>
     </row>
     <row r="647" spans="1:7">
@@ -19879,7 +19876,7 @@
         <v>1133</v>
       </c>
       <c r="G647" t="s">
-        <v>1318</v>
+        <v>1317</v>
       </c>
     </row>
     <row r="648" spans="1:7">
@@ -19903,7 +19900,7 @@
         <v>1130</v>
       </c>
       <c r="G648" t="s">
-        <v>1319</v>
+        <v>1318</v>
       </c>
     </row>
     <row r="649" spans="1:7">
@@ -19927,7 +19924,7 @@
         <v>1133</v>
       </c>
       <c r="G649" t="s">
-        <v>1318</v>
+        <v>1317</v>
       </c>
     </row>
     <row r="650" spans="1:7">
@@ -19951,7 +19948,7 @@
         <v>1130</v>
       </c>
       <c r="G650" t="s">
-        <v>1319</v>
+        <v>1318</v>
       </c>
     </row>
     <row r="651" spans="1:7">
@@ -19975,7 +19972,7 @@
         <v>1133</v>
       </c>
       <c r="G651" t="s">
-        <v>1318</v>
+        <v>1317</v>
       </c>
     </row>
     <row r="652" spans="1:7">
@@ -19999,7 +19996,7 @@
         <v>1130</v>
       </c>
       <c r="G652" t="s">
-        <v>1319</v>
+        <v>1318</v>
       </c>
     </row>
     <row r="653" spans="1:7">
@@ -20023,7 +20020,7 @@
         <v>1133</v>
       </c>
       <c r="G653" t="s">
-        <v>1318</v>
+        <v>1317</v>
       </c>
     </row>
     <row r="654" spans="1:7">
@@ -20047,7 +20044,7 @@
         <v>1130</v>
       </c>
       <c r="G654" t="s">
-        <v>1319</v>
+        <v>1318</v>
       </c>
     </row>
     <row r="655" spans="1:7">
@@ -20095,7 +20092,7 @@
         <v>1123</v>
       </c>
       <c r="G656" t="s">
-        <v>1320</v>
+        <v>1319</v>
       </c>
     </row>
     <row r="657" spans="1:7">
@@ -20119,7 +20116,7 @@
         <v>1123</v>
       </c>
       <c r="G657" t="s">
-        <v>1321</v>
+        <v>1320</v>
       </c>
     </row>
     <row r="658" spans="1:7">
@@ -20143,7 +20140,7 @@
         <v>1123</v>
       </c>
       <c r="G658" t="s">
-        <v>1322</v>
+        <v>1321</v>
       </c>
     </row>
     <row r="659" spans="1:7">
@@ -20167,7 +20164,7 @@
         <v>1123</v>
       </c>
       <c r="G659" t="s">
-        <v>1323</v>
+        <v>1322</v>
       </c>
     </row>
     <row r="660" spans="1:7">
@@ -20191,7 +20188,7 @@
         <v>1123</v>
       </c>
       <c r="G660" t="s">
-        <v>1324</v>
+        <v>1323</v>
       </c>
     </row>
     <row r="661" spans="1:7">
@@ -20215,7 +20212,7 @@
         <v>1125</v>
       </c>
       <c r="G661" t="s">
-        <v>1325</v>
+        <v>1324</v>
       </c>
     </row>
     <row r="662" spans="1:7">
@@ -20309,7 +20306,7 @@
         <v>1125</v>
       </c>
       <c r="G665" t="s">
-        <v>1325</v>
+        <v>1324</v>
       </c>
     </row>
     <row r="666" spans="1:7">
@@ -20403,7 +20400,7 @@
         <v>1125</v>
       </c>
       <c r="G669" t="s">
-        <v>1325</v>
+        <v>1324</v>
       </c>
     </row>
     <row r="670" spans="1:7">
@@ -20497,7 +20494,7 @@
         <v>1123</v>
       </c>
       <c r="G673" t="s">
-        <v>1326</v>
+        <v>1325</v>
       </c>
     </row>
     <row r="674" spans="1:7">
@@ -20521,7 +20518,7 @@
         <v>1125</v>
       </c>
       <c r="G674" t="s">
-        <v>1327</v>
+        <v>1326</v>
       </c>
     </row>
     <row r="675" spans="1:7">
@@ -20569,7 +20566,7 @@
         <v>1123</v>
       </c>
       <c r="G676" t="s">
-        <v>1328</v>
+        <v>1327</v>
       </c>
     </row>
     <row r="677" spans="1:7">
@@ -21216,7 +21213,7 @@
         <v>1125</v>
       </c>
       <c r="G703" t="s">
-        <v>1329</v>
+        <v>1328</v>
       </c>
     </row>
     <row r="704" spans="1:7">
@@ -21333,7 +21330,7 @@
         <v>1125</v>
       </c>
       <c r="G708" t="s">
-        <v>1330</v>
+        <v>1329</v>
       </c>
     </row>
     <row r="709" spans="1:7">
@@ -21452,7 +21449,7 @@
         <v>1125</v>
       </c>
       <c r="G713" t="s">
-        <v>1331</v>
+        <v>1330</v>
       </c>
     </row>
     <row r="714" spans="1:7">
@@ -21690,7 +21687,7 @@
         <v>1125</v>
       </c>
       <c r="G723" t="s">
-        <v>1332</v>
+        <v>1331</v>
       </c>
     </row>
     <row r="724" spans="1:7">
@@ -22094,7 +22091,7 @@
         <v>1125</v>
       </c>
       <c r="G740" t="s">
-        <v>1333</v>
+        <v>1332</v>
       </c>
     </row>
     <row r="741" spans="1:7">
@@ -22499,7 +22496,7 @@
         <v>1125</v>
       </c>
       <c r="G757" t="s">
-        <v>1334</v>
+        <v>1333</v>
       </c>
     </row>
     <row r="758" spans="1:7">
@@ -22547,7 +22544,7 @@
         <v>1125</v>
       </c>
       <c r="G759" t="s">
-        <v>1335</v>
+        <v>1334</v>
       </c>
     </row>
     <row r="760" spans="1:7">
@@ -22595,7 +22592,7 @@
         <v>1125</v>
       </c>
       <c r="G761" t="s">
-        <v>1336</v>
+        <v>1335</v>
       </c>
     </row>
     <row r="762" spans="1:7">
@@ -22613,7 +22610,7 @@
         <v>0</v>
       </c>
       <c r="E762" t="s">
-        <v>1124</v>
+        <v>1121</v>
       </c>
       <c r="F762" t="s">
         <v>1123</v>
@@ -22667,7 +22664,7 @@
         <v>1125</v>
       </c>
       <c r="G764" t="s">
-        <v>1337</v>
+        <v>1336</v>
       </c>
     </row>
     <row r="765" spans="1:7">
@@ -22739,7 +22736,7 @@
         <v>1125</v>
       </c>
       <c r="G767" t="s">
-        <v>1338</v>
+        <v>1337</v>
       </c>
     </row>
     <row r="768" spans="1:7">
@@ -22811,7 +22808,7 @@
         <v>1125</v>
       </c>
       <c r="G770" t="s">
-        <v>1339</v>
+        <v>1338</v>
       </c>
     </row>
     <row r="771" spans="1:7">
@@ -22829,7 +22826,7 @@
         <v>0</v>
       </c>
       <c r="E771" t="s">
-        <v>1124</v>
+        <v>1121</v>
       </c>
       <c r="F771" t="s">
         <v>1123</v>
@@ -23050,7 +23047,7 @@
         <v>1123</v>
       </c>
       <c r="G780" t="s">
-        <v>1340</v>
+        <v>1339</v>
       </c>
     </row>
     <row r="781" spans="1:7">
@@ -23472,17 +23469,17 @@
         <v>1064</v>
       </c>
       <c r="D798">
-        <f>1</f>
+        <f>1/1.23</f>
         <v>0</v>
       </c>
       <c r="E798" t="s">
-        <v>1126</v>
+        <v>1127</v>
       </c>
       <c r="F798" t="s">
         <v>1126</v>
       </c>
       <c r="G798" t="s">
-        <v>1137</v>
+        <v>1158</v>
       </c>
     </row>
     <row r="799" spans="1:7">
@@ -23520,17 +23517,17 @@
         <v>1065</v>
       </c>
       <c r="D800">
-        <f>1</f>
+        <f>1/1.23</f>
         <v>0</v>
       </c>
       <c r="E800" t="s">
-        <v>1126</v>
+        <v>1127</v>
       </c>
       <c r="F800" t="s">
         <v>1126</v>
       </c>
       <c r="G800" t="s">
-        <v>1137</v>
+        <v>1158</v>
       </c>
     </row>
     <row r="801" spans="1:7">
@@ -23568,17 +23565,17 @@
         <v>1066</v>
       </c>
       <c r="D802">
-        <f>1</f>
+        <f>1/1.23</f>
         <v>0</v>
       </c>
       <c r="E802" t="s">
-        <v>1126</v>
+        <v>1127</v>
       </c>
       <c r="F802" t="s">
         <v>1126</v>
       </c>
       <c r="G802" t="s">
-        <v>1137</v>
+        <v>1158</v>
       </c>
     </row>
     <row r="803" spans="1:7">
@@ -23602,7 +23599,7 @@
         <v>1132</v>
       </c>
       <c r="G803" t="s">
-        <v>1312</v>
+        <v>1311</v>
       </c>
     </row>
     <row r="804" spans="1:7">
@@ -23650,7 +23647,7 @@
         <v>1133</v>
       </c>
       <c r="G805" t="s">
-        <v>1313</v>
+        <v>1312</v>
       </c>
     </row>
     <row r="806" spans="1:7">
@@ -23697,7 +23694,7 @@
         <v>1133</v>
       </c>
       <c r="G807" t="s">
-        <v>1313</v>
+        <v>1312</v>
       </c>
     </row>
     <row r="808" spans="1:7">
@@ -23744,7 +23741,7 @@
         <v>1132</v>
       </c>
       <c r="G809" t="s">
-        <v>1312</v>
+        <v>1311</v>
       </c>
     </row>
     <row r="810" spans="1:7">
@@ -23792,7 +23789,7 @@
         <v>1133</v>
       </c>
       <c r="G811" t="s">
-        <v>1316</v>
+        <v>1315</v>
       </c>
     </row>
     <row r="812" spans="1:7">
@@ -23816,7 +23813,7 @@
         <v>1130</v>
       </c>
       <c r="G812" t="s">
-        <v>1317</v>
+        <v>1316</v>
       </c>
     </row>
     <row r="813" spans="1:7">
@@ -23840,7 +23837,7 @@
         <v>1133</v>
       </c>
       <c r="G813" t="s">
-        <v>1318</v>
+        <v>1317</v>
       </c>
     </row>
     <row r="814" spans="1:7">
@@ -23864,7 +23861,7 @@
         <v>1130</v>
       </c>
       <c r="G814" t="s">
-        <v>1319</v>
+        <v>1318</v>
       </c>
     </row>
     <row r="815" spans="1:7">
@@ -23912,7 +23909,7 @@
         <v>1125</v>
       </c>
       <c r="G816" t="s">
-        <v>1341</v>
+        <v>1340</v>
       </c>
     </row>
     <row r="817" spans="1:7">
@@ -23936,7 +23933,7 @@
         <v>1125</v>
       </c>
       <c r="G817" t="s">
-        <v>1342</v>
+        <v>1341</v>
       </c>
     </row>
     <row r="818" spans="1:7">
@@ -23960,7 +23957,7 @@
         <v>1125</v>
       </c>
       <c r="G818" t="s">
-        <v>1343</v>
+        <v>1342</v>
       </c>
     </row>
     <row r="819" spans="1:7">
@@ -23984,7 +23981,7 @@
         <v>1125</v>
       </c>
       <c r="G819" t="s">
-        <v>1344</v>
+        <v>1343</v>
       </c>
     </row>
     <row r="820" spans="1:7">
@@ -24008,7 +24005,7 @@
         <v>1125</v>
       </c>
       <c r="G820" t="s">
-        <v>1345</v>
+        <v>1344</v>
       </c>
     </row>
     <row r="821" spans="1:7">
@@ -24032,7 +24029,7 @@
         <v>1125</v>
       </c>
       <c r="G821" t="s">
-        <v>1346</v>
+        <v>1345</v>
       </c>
     </row>
     <row r="822" spans="1:7">
@@ -24056,7 +24053,7 @@
         <v>1125</v>
       </c>
       <c r="G822" t="s">
-        <v>1347</v>
+        <v>1346</v>
       </c>
     </row>
     <row r="823" spans="1:7">
@@ -24080,7 +24077,7 @@
         <v>1125</v>
       </c>
       <c r="G823" t="s">
-        <v>1348</v>
+        <v>1347</v>
       </c>
     </row>
     <row r="824" spans="1:7">
@@ -24670,7 +24667,7 @@
         <v>839</v>
       </c>
       <c r="D848">
-        <f>1 / (0.777 * 13.1)</f>
+        <f>1 * 3.6 / 39</f>
         <v>0</v>
       </c>
       <c r="E848" t="s">
@@ -24694,7 +24691,7 @@
         <v>839</v>
       </c>
       <c r="D849">
-        <f>1 / (0.777 * 13.1)</f>
+        <f>1 * 3.6 / 39</f>
         <v>0</v>
       </c>
       <c r="E849" t="s">
@@ -24718,17 +24715,17 @@
         <v>839</v>
       </c>
       <c r="D850">
-        <f>1 / (0.777 * 13.1)</f>
+        <f>1 * 3.6 / 46.5</f>
         <v>0</v>
       </c>
       <c r="E850" t="s">
-        <v>1124</v>
+        <v>1121</v>
       </c>
       <c r="F850" t="s">
         <v>1123</v>
       </c>
       <c r="G850" t="s">
-        <v>1274</v>
+        <v>1277</v>
       </c>
     </row>
     <row r="851" spans="1:7">
@@ -24925,64 +24922,64 @@
     </row>
     <row r="859" spans="1:7">
       <c r="A859" t="s">
-        <v>357</v>
+        <v>368</v>
       </c>
       <c r="B859" t="s">
         <v>570</v>
       </c>
       <c r="C859" t="s">
-        <v>914</v>
+        <v>925</v>
       </c>
       <c r="D859">
-        <f>1 / (0.777 * 13.1)</f>
+        <f>1</f>
         <v>0</v>
       </c>
       <c r="E859" t="s">
-        <v>1124</v>
+        <v>1121</v>
       </c>
       <c r="F859" t="s">
-        <v>1123</v>
+        <v>1121</v>
       </c>
       <c r="G859" t="s">
-        <v>1307</v>
+        <v>1137</v>
       </c>
     </row>
     <row r="860" spans="1:7">
       <c r="A860" t="s">
-        <v>368</v>
+        <v>383</v>
       </c>
       <c r="B860" t="s">
         <v>570</v>
       </c>
       <c r="C860" t="s">
-        <v>925</v>
+        <v>940</v>
       </c>
       <c r="D860">
-        <f>1</f>
+        <f>1 * 3.6 / 42.43</f>
         <v>0</v>
       </c>
       <c r="E860" t="s">
         <v>1121</v>
       </c>
       <c r="F860" t="s">
-        <v>1121</v>
+        <v>1123</v>
       </c>
       <c r="G860" t="s">
-        <v>1137</v>
+        <v>1310</v>
       </c>
     </row>
     <row r="861" spans="1:7">
       <c r="A861" t="s">
-        <v>383</v>
+        <v>417</v>
       </c>
       <c r="B861" t="s">
         <v>570</v>
       </c>
       <c r="C861" t="s">
-        <v>940</v>
+        <v>974</v>
       </c>
       <c r="D861">
-        <f>1 * 3.6 / 42.43</f>
+        <f>1 * 3.6 / (3900*1000)</f>
         <v>0</v>
       </c>
       <c r="E861" t="s">
@@ -24992,21 +24989,21 @@
         <v>1123</v>
       </c>
       <c r="G861" t="s">
-        <v>1311</v>
+        <v>1319</v>
       </c>
     </row>
     <row r="862" spans="1:7">
       <c r="A862" t="s">
-        <v>417</v>
+        <v>418</v>
       </c>
       <c r="B862" t="s">
         <v>570</v>
       </c>
       <c r="C862" t="s">
-        <v>974</v>
+        <v>975</v>
       </c>
       <c r="D862">
-        <f>1 * 3.6 / (3900*1000)</f>
+        <f>-1 * 3.6 / 12.35</f>
         <v>0</v>
       </c>
       <c r="E862" t="s">
@@ -25021,16 +25018,16 @@
     </row>
     <row r="863" spans="1:7">
       <c r="A863" t="s">
-        <v>418</v>
+        <v>419</v>
       </c>
       <c r="B863" t="s">
         <v>570</v>
       </c>
       <c r="C863" t="s">
-        <v>975</v>
+        <v>976</v>
       </c>
       <c r="D863">
-        <f>-1 * 3.6 / 12.35</f>
+        <f>-1 * 3.6 / (6.087*0.95)</f>
         <v>0</v>
       </c>
       <c r="E863" t="s">
@@ -25045,16 +25042,16 @@
     </row>
     <row r="864" spans="1:7">
       <c r="A864" t="s">
-        <v>419</v>
+        <v>420</v>
       </c>
       <c r="B864" t="s">
         <v>570</v>
       </c>
       <c r="C864" t="s">
-        <v>976</v>
+        <v>977</v>
       </c>
       <c r="D864">
-        <f>-1 * 3.6 / (6.087*0.95)</f>
+        <f>-1 * 3.6 / 2.453</f>
         <v>0</v>
       </c>
       <c r="E864" t="s">
@@ -25069,16 +25066,16 @@
     </row>
     <row r="865" spans="1:7">
       <c r="A865" t="s">
-        <v>420</v>
+        <v>421</v>
       </c>
       <c r="B865" t="s">
         <v>570</v>
       </c>
       <c r="C865" t="s">
-        <v>977</v>
+        <v>978</v>
       </c>
       <c r="D865">
-        <f>-1 * 3.6 / 2.453</f>
+        <f>1 * 3.6 / (0.95*15)</f>
         <v>0</v>
       </c>
       <c r="E865" t="s">
@@ -25093,16 +25090,16 @@
     </row>
     <row r="866" spans="1:7">
       <c r="A866" t="s">
-        <v>421</v>
+        <v>431</v>
       </c>
       <c r="B866" t="s">
         <v>570</v>
       </c>
       <c r="C866" t="s">
-        <v>978</v>
+        <v>988</v>
       </c>
       <c r="D866">
-        <f>1 * 3.6 / (0.95*15)</f>
+        <f>1 * 3.6 / 15.4</f>
         <v>0</v>
       </c>
       <c r="E866" t="s">
@@ -25112,21 +25109,21 @@
         <v>1123</v>
       </c>
       <c r="G866" t="s">
-        <v>1324</v>
+        <v>1325</v>
       </c>
     </row>
     <row r="867" spans="1:7">
       <c r="A867" t="s">
-        <v>431</v>
+        <v>433</v>
       </c>
       <c r="B867" t="s">
         <v>570</v>
       </c>
       <c r="C867" t="s">
-        <v>988</v>
+        <v>990</v>
       </c>
       <c r="D867">
-        <f>1 * 3.6 / 15.4</f>
+        <f>1 * 3.6 / 40.961</f>
         <v>0</v>
       </c>
       <c r="E867" t="s">
@@ -25136,21 +25133,21 @@
         <v>1123</v>
       </c>
       <c r="G867" t="s">
-        <v>1326</v>
+        <v>1327</v>
       </c>
     </row>
     <row r="868" spans="1:7">
       <c r="A868" t="s">
-        <v>433</v>
+        <v>516</v>
       </c>
       <c r="B868" t="s">
         <v>570</v>
       </c>
       <c r="C868" t="s">
-        <v>990</v>
+        <v>1073</v>
       </c>
       <c r="D868">
-        <f>1 * 3.6 / 40.961</f>
+        <f>1 * 3.6 / 31.58</f>
         <v>0</v>
       </c>
       <c r="E868" t="s">
@@ -25160,21 +25157,21 @@
         <v>1123</v>
       </c>
       <c r="G868" t="s">
-        <v>1328</v>
+        <v>1218</v>
       </c>
     </row>
     <row r="869" spans="1:7">
       <c r="A869" t="s">
-        <v>516</v>
+        <v>528</v>
       </c>
       <c r="B869" t="s">
         <v>570</v>
       </c>
       <c r="C869" t="s">
-        <v>1073</v>
+        <v>1085</v>
       </c>
       <c r="D869">
-        <f>1 * 3.6 / 31.58</f>
+        <f>1 * 3.6 / 43</f>
         <v>0</v>
       </c>
       <c r="E869" t="s">
@@ -25184,21 +25181,21 @@
         <v>1123</v>
       </c>
       <c r="G869" t="s">
-        <v>1218</v>
+        <v>1175</v>
       </c>
     </row>
     <row r="870" spans="1:7">
       <c r="A870" t="s">
-        <v>528</v>
+        <v>529</v>
       </c>
       <c r="B870" t="s">
         <v>570</v>
       </c>
       <c r="C870" t="s">
-        <v>1085</v>
+        <v>1086</v>
       </c>
       <c r="D870">
-        <f>1 * 3.6 / 43</f>
+        <f>1 * 3.6 / 42.6</f>
         <v>0</v>
       </c>
       <c r="E870" t="s">
@@ -25208,21 +25205,21 @@
         <v>1123</v>
       </c>
       <c r="G870" t="s">
-        <v>1175</v>
+        <v>1259</v>
       </c>
     </row>
     <row r="871" spans="1:7">
       <c r="A871" t="s">
-        <v>529</v>
+        <v>530</v>
       </c>
       <c r="B871" t="s">
         <v>570</v>
       </c>
       <c r="C871" t="s">
-        <v>1086</v>
+        <v>1087</v>
       </c>
       <c r="D871">
-        <f>1 * 3.6 / 42.6</f>
+        <f>1 / 5.54</f>
         <v>0</v>
       </c>
       <c r="E871" t="s">
@@ -25232,36 +25229,36 @@
         <v>1123</v>
       </c>
       <c r="G871" t="s">
-        <v>1259</v>
+        <v>1267</v>
       </c>
     </row>
     <row r="872" spans="1:7">
       <c r="A872" t="s">
-        <v>530</v>
+        <v>357</v>
       </c>
       <c r="B872" t="s">
         <v>570</v>
       </c>
       <c r="C872" t="s">
-        <v>1087</v>
+        <v>914</v>
       </c>
       <c r="D872">
-        <f>1 / 5.54</f>
+        <f>1 * 3.6 / 39</f>
         <v>0</v>
       </c>
       <c r="E872" t="s">
-        <v>1121</v>
+        <v>1124</v>
       </c>
       <c r="F872" t="s">
         <v>1123</v>
       </c>
       <c r="G872" t="s">
-        <v>1267</v>
+        <v>1274</v>
       </c>
     </row>
     <row r="873" spans="1:7">
       <c r="A873" t="s">
-        <v>357</v>
+        <v>531</v>
       </c>
       <c r="B873" t="s">
         <v>570</v>
@@ -25270,7 +25267,7 @@
         <v>914</v>
       </c>
       <c r="D873">
-        <f>1 * 3.6 / 39</f>
+        <f>1 / (0.777 * 13.1)</f>
         <v>0</v>
       </c>
       <c r="E873" t="s">
@@ -25285,7 +25282,7 @@
     </row>
     <row r="874" spans="1:7">
       <c r="A874" t="s">
-        <v>531</v>
+        <v>532</v>
       </c>
       <c r="B874" t="s">
         <v>570</v>
@@ -25309,7 +25306,7 @@
     </row>
     <row r="875" spans="1:7">
       <c r="A875" t="s">
-        <v>532</v>
+        <v>533</v>
       </c>
       <c r="B875" t="s">
         <v>570</v>
@@ -25333,37 +25330,37 @@
     </row>
     <row r="876" spans="1:7">
       <c r="A876" t="s">
-        <v>533</v>
+        <v>534</v>
       </c>
       <c r="B876" t="s">
         <v>570</v>
       </c>
       <c r="C876" t="s">
-        <v>914</v>
+        <v>1088</v>
       </c>
       <c r="D876">
-        <f>1 / (0.777 * 13.1)</f>
+        <f>1 * 3.6</f>
         <v>0</v>
       </c>
       <c r="E876" t="s">
-        <v>1124</v>
+        <v>1128</v>
       </c>
       <c r="F876" t="s">
         <v>1123</v>
       </c>
       <c r="G876" t="s">
-        <v>1274</v>
+        <v>1137</v>
       </c>
     </row>
     <row r="877" spans="1:7">
       <c r="A877" t="s">
-        <v>534</v>
+        <v>535</v>
       </c>
       <c r="B877" t="s">
         <v>570</v>
       </c>
       <c r="C877" t="s">
-        <v>1088</v>
+        <v>1089</v>
       </c>
       <c r="D877">
         <f>1 * 3.6</f>
@@ -25381,23 +25378,22 @@
     </row>
     <row r="878" spans="1:7">
       <c r="A878" t="s">
-        <v>535</v>
+        <v>536</v>
       </c>
       <c r="B878" t="s">
         <v>570</v>
       </c>
       <c r="C878" t="s">
-        <v>1089</v>
+        <v>1090</v>
       </c>
       <c r="D878">
-        <f>1 * 3.6</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E878" t="s">
-        <v>1128</v>
+        <v>1121</v>
       </c>
       <c r="F878" t="s">
-        <v>1123</v>
+        <v>1121</v>
       </c>
       <c r="G878" t="s">
         <v>1137</v>
@@ -25405,39 +25401,40 @@
     </row>
     <row r="879" spans="1:7">
       <c r="A879" t="s">
-        <v>536</v>
+        <v>537</v>
       </c>
       <c r="B879" t="s">
-        <v>570</v>
+        <v>567</v>
       </c>
       <c r="C879" t="s">
-        <v>1090</v>
+        <v>1091</v>
       </c>
       <c r="D879">
-        <v>1</v>
+        <f>3.6/18.43</f>
+        <v>0</v>
       </c>
       <c r="E879" t="s">
         <v>1121</v>
       </c>
       <c r="F879" t="s">
-        <v>1121</v>
+        <v>1123</v>
       </c>
       <c r="G879" t="s">
-        <v>1137</v>
+        <v>1348</v>
       </c>
     </row>
     <row r="880" spans="1:7">
       <c r="A880" t="s">
-        <v>537</v>
+        <v>538</v>
       </c>
       <c r="B880" t="s">
         <v>567</v>
       </c>
       <c r="C880" t="s">
-        <v>1091</v>
+        <v>1092</v>
       </c>
       <c r="D880">
-        <f>3.6/18.43</f>
+        <f>3.6/18.61</f>
         <v>0</v>
       </c>
       <c r="E880" t="s">
@@ -25452,16 +25449,16 @@
     </row>
     <row r="881" spans="1:7">
       <c r="A881" t="s">
-        <v>538</v>
+        <v>539</v>
       </c>
       <c r="B881" t="s">
         <v>567</v>
       </c>
       <c r="C881" t="s">
-        <v>1092</v>
+        <v>1093</v>
       </c>
       <c r="D881">
-        <f>3.6/18.61</f>
+        <f>3.6/19.06</f>
         <v>0</v>
       </c>
       <c r="E881" t="s">
@@ -25476,16 +25473,16 @@
     </row>
     <row r="882" spans="1:7">
       <c r="A882" t="s">
-        <v>539</v>
+        <v>540</v>
       </c>
       <c r="B882" t="s">
         <v>567</v>
       </c>
       <c r="C882" t="s">
-        <v>1093</v>
+        <v>1094</v>
       </c>
       <c r="D882">
-        <f>3.6/19.06</f>
+        <f>3.6/18.93</f>
         <v>0</v>
       </c>
       <c r="E882" t="s">
@@ -25500,16 +25497,16 @@
     </row>
     <row r="883" spans="1:7">
       <c r="A883" t="s">
-        <v>540</v>
+        <v>541</v>
       </c>
       <c r="B883" t="s">
         <v>567</v>
       </c>
       <c r="C883" t="s">
-        <v>1094</v>
+        <v>1095</v>
       </c>
       <c r="D883">
-        <f>3.6/18.93</f>
+        <f>3.6 / 7.09</f>
         <v>0</v>
       </c>
       <c r="E883" t="s">
@@ -25524,16 +25521,16 @@
     </row>
     <row r="884" spans="1:7">
       <c r="A884" t="s">
-        <v>541</v>
+        <v>542</v>
       </c>
       <c r="B884" t="s">
         <v>567</v>
       </c>
       <c r="C884" t="s">
-        <v>1095</v>
+        <v>1096</v>
       </c>
       <c r="D884">
-        <f>3.6 / 7.09</f>
+        <f>3.6/15.34</f>
         <v>0</v>
       </c>
       <c r="E884" t="s">
@@ -25548,16 +25545,16 @@
     </row>
     <row r="885" spans="1:7">
       <c r="A885" t="s">
-        <v>542</v>
+        <v>543</v>
       </c>
       <c r="B885" t="s">
         <v>567</v>
       </c>
       <c r="C885" t="s">
-        <v>1096</v>
+        <v>1097</v>
       </c>
       <c r="D885">
-        <f>3.6/15.34</f>
+        <f>-1 * 3.6 / 17.09</f>
         <v>0</v>
       </c>
       <c r="E885" t="s">
@@ -25572,16 +25569,16 @@
     </row>
     <row r="886" spans="1:7">
       <c r="A886" t="s">
-        <v>543</v>
+        <v>544</v>
       </c>
       <c r="B886" t="s">
         <v>567</v>
       </c>
       <c r="C886" t="s">
-        <v>1097</v>
+        <v>1098</v>
       </c>
       <c r="D886">
-        <f>-1 * 3.6 / 17.09</f>
+        <f>3.6/15.98</f>
         <v>0</v>
       </c>
       <c r="E886" t="s">
@@ -25596,16 +25593,16 @@
     </row>
     <row r="887" spans="1:7">
       <c r="A887" t="s">
-        <v>544</v>
+        <v>545</v>
       </c>
       <c r="B887" t="s">
         <v>567</v>
       </c>
       <c r="C887" t="s">
-        <v>1098</v>
+        <v>1099</v>
       </c>
       <c r="D887">
-        <f>3.6/15.98</f>
+        <f>-1 * 3.6 / 11.24</f>
         <v>0</v>
       </c>
       <c r="E887" t="s">
@@ -25620,16 +25617,16 @@
     </row>
     <row r="888" spans="1:7">
       <c r="A888" t="s">
-        <v>545</v>
+        <v>546</v>
       </c>
       <c r="B888" t="s">
         <v>567</v>
       </c>
       <c r="C888" t="s">
-        <v>1099</v>
+        <v>1100</v>
       </c>
       <c r="D888">
-        <f>-1 * 3.6 / 11.24</f>
+        <f>3.6/18.63</f>
         <v>0</v>
       </c>
       <c r="E888" t="s">
@@ -25644,16 +25641,16 @@
     </row>
     <row r="889" spans="1:7">
       <c r="A889" t="s">
-        <v>546</v>
+        <v>547</v>
       </c>
       <c r="B889" t="s">
         <v>567</v>
       </c>
       <c r="C889" t="s">
-        <v>1100</v>
+        <v>1101</v>
       </c>
       <c r="D889">
-        <f>3.6/18.63</f>
+        <f>-1 * 3.6 / 7.64</f>
         <v>0</v>
       </c>
       <c r="E889" t="s">
@@ -25668,16 +25665,16 @@
     </row>
     <row r="890" spans="1:7">
       <c r="A890" t="s">
-        <v>547</v>
+        <v>537</v>
       </c>
       <c r="B890" t="s">
-        <v>567</v>
+        <v>570</v>
       </c>
       <c r="C890" t="s">
-        <v>1101</v>
+        <v>1091</v>
       </c>
       <c r="D890">
-        <f>-1 * 3.6 / 7.64</f>
+        <f>3.6/18.43</f>
         <v>0</v>
       </c>
       <c r="E890" t="s">
@@ -25687,21 +25684,21 @@
         <v>1123</v>
       </c>
       <c r="G890" t="s">
-        <v>1359</v>
+        <v>1348</v>
       </c>
     </row>
     <row r="891" spans="1:7">
       <c r="A891" t="s">
-        <v>537</v>
+        <v>538</v>
       </c>
       <c r="B891" t="s">
         <v>570</v>
       </c>
       <c r="C891" t="s">
-        <v>1091</v>
+        <v>1092</v>
       </c>
       <c r="D891">
-        <f>3.6/18.43</f>
+        <f>3.6/18.61</f>
         <v>0</v>
       </c>
       <c r="E891" t="s">
@@ -25716,16 +25713,16 @@
     </row>
     <row r="892" spans="1:7">
       <c r="A892" t="s">
-        <v>538</v>
+        <v>539</v>
       </c>
       <c r="B892" t="s">
         <v>570</v>
       </c>
       <c r="C892" t="s">
-        <v>1092</v>
+        <v>1093</v>
       </c>
       <c r="D892">
-        <f>3.6/18.61</f>
+        <f>3.6/19.06</f>
         <v>0</v>
       </c>
       <c r="E892" t="s">
@@ -25740,16 +25737,16 @@
     </row>
     <row r="893" spans="1:7">
       <c r="A893" t="s">
-        <v>539</v>
+        <v>540</v>
       </c>
       <c r="B893" t="s">
         <v>570</v>
       </c>
       <c r="C893" t="s">
-        <v>1093</v>
+        <v>1094</v>
       </c>
       <c r="D893">
-        <f>3.6/19.06</f>
+        <f>3.6/18.93</f>
         <v>0</v>
       </c>
       <c r="E893" t="s">
@@ -25764,16 +25761,16 @@
     </row>
     <row r="894" spans="1:7">
       <c r="A894" t="s">
-        <v>540</v>
+        <v>541</v>
       </c>
       <c r="B894" t="s">
         <v>570</v>
       </c>
       <c r="C894" t="s">
-        <v>1094</v>
+        <v>1095</v>
       </c>
       <c r="D894">
-        <f>3.6/18.93</f>
+        <f>3.6 / 7.09</f>
         <v>0</v>
       </c>
       <c r="E894" t="s">
@@ -25788,16 +25785,16 @@
     </row>
     <row r="895" spans="1:7">
       <c r="A895" t="s">
-        <v>541</v>
+        <v>542</v>
       </c>
       <c r="B895" t="s">
         <v>570</v>
       </c>
       <c r="C895" t="s">
-        <v>1095</v>
+        <v>1096</v>
       </c>
       <c r="D895">
-        <f>3.6 / 7.09</f>
+        <f>3.6/15.34</f>
         <v>0</v>
       </c>
       <c r="E895" t="s">
@@ -25812,16 +25809,16 @@
     </row>
     <row r="896" spans="1:7">
       <c r="A896" t="s">
-        <v>542</v>
+        <v>543</v>
       </c>
       <c r="B896" t="s">
         <v>570</v>
       </c>
       <c r="C896" t="s">
-        <v>1096</v>
+        <v>1097</v>
       </c>
       <c r="D896">
-        <f>3.6/15.34</f>
+        <f>-1 * 3.6 / 17.09</f>
         <v>0</v>
       </c>
       <c r="E896" t="s">
@@ -25836,16 +25833,16 @@
     </row>
     <row r="897" spans="1:7">
       <c r="A897" t="s">
-        <v>543</v>
+        <v>544</v>
       </c>
       <c r="B897" t="s">
         <v>570</v>
       </c>
       <c r="C897" t="s">
-        <v>1097</v>
+        <v>1098</v>
       </c>
       <c r="D897">
-        <f>-1 * 3.6 / 17.09</f>
+        <f>3.6/15.98</f>
         <v>0</v>
       </c>
       <c r="E897" t="s">
@@ -25860,16 +25857,16 @@
     </row>
     <row r="898" spans="1:7">
       <c r="A898" t="s">
-        <v>544</v>
+        <v>545</v>
       </c>
       <c r="B898" t="s">
         <v>570</v>
       </c>
       <c r="C898" t="s">
-        <v>1098</v>
+        <v>1099</v>
       </c>
       <c r="D898">
-        <f>3.6/15.98</f>
+        <f>-1 * 3.6 / 11.24</f>
         <v>0</v>
       </c>
       <c r="E898" t="s">
@@ -25884,16 +25881,16 @@
     </row>
     <row r="899" spans="1:7">
       <c r="A899" t="s">
-        <v>545</v>
+        <v>546</v>
       </c>
       <c r="B899" t="s">
         <v>570</v>
       </c>
       <c r="C899" t="s">
-        <v>1099</v>
+        <v>1100</v>
       </c>
       <c r="D899">
-        <f>-1 * 3.6 / 11.24</f>
+        <f>3.6/18.63</f>
         <v>0</v>
       </c>
       <c r="E899" t="s">
@@ -25908,16 +25905,16 @@
     </row>
     <row r="900" spans="1:7">
       <c r="A900" t="s">
-        <v>546</v>
+        <v>547</v>
       </c>
       <c r="B900" t="s">
         <v>570</v>
       </c>
       <c r="C900" t="s">
-        <v>1100</v>
+        <v>1101</v>
       </c>
       <c r="D900">
-        <f>3.6/18.63</f>
+        <f>-1 * 3.6 / 7.64</f>
         <v>0</v>
       </c>
       <c r="E900" t="s">
@@ -25932,16 +25929,16 @@
     </row>
     <row r="901" spans="1:7">
       <c r="A901" t="s">
-        <v>547</v>
+        <v>548</v>
       </c>
       <c r="B901" t="s">
-        <v>570</v>
+        <v>567</v>
       </c>
       <c r="C901" t="s">
-        <v>1101</v>
+        <v>1102</v>
       </c>
       <c r="D901">
-        <f>-1 * 3.6 / 7.64</f>
+        <f>1/10.83</f>
         <v>0</v>
       </c>
       <c r="E901" t="s">
@@ -25959,7 +25956,7 @@
         <v>548</v>
       </c>
       <c r="B902" t="s">
-        <v>567</v>
+        <v>570</v>
       </c>
       <c r="C902" t="s">
         <v>1102</v>
@@ -25975,18 +25972,18 @@
         <v>1123</v>
       </c>
       <c r="G902" t="s">
-        <v>1360</v>
+        <v>1359</v>
       </c>
     </row>
     <row r="903" spans="1:7">
       <c r="A903" t="s">
-        <v>548</v>
+        <v>549</v>
       </c>
       <c r="B903" t="s">
-        <v>570</v>
+        <v>567</v>
       </c>
       <c r="C903" t="s">
-        <v>1102</v>
+        <v>1103</v>
       </c>
       <c r="D903">
         <f>1/10.83</f>
@@ -25999,7 +25996,7 @@
         <v>1123</v>
       </c>
       <c r="G903" t="s">
-        <v>1360</v>
+        <v>1359</v>
       </c>
     </row>
     <row r="904" spans="1:7">
@@ -26007,7 +26004,7 @@
         <v>549</v>
       </c>
       <c r="B904" t="s">
-        <v>567</v>
+        <v>570</v>
       </c>
       <c r="C904" t="s">
         <v>1103</v>
@@ -26023,28 +26020,28 @@
         <v>1123</v>
       </c>
       <c r="G904" t="s">
-        <v>1360</v>
+        <v>1359</v>
       </c>
     </row>
     <row r="905" spans="1:7">
       <c r="A905" t="s">
-        <v>549</v>
+        <v>550</v>
       </c>
       <c r="B905" t="s">
-        <v>570</v>
+        <v>568</v>
       </c>
       <c r="C905" t="s">
-        <v>1103</v>
+        <v>1104</v>
       </c>
       <c r="D905">
-        <f>1/10.83</f>
+        <f>8760 * 0.7 / (7200 * 1000000)</f>
         <v>0</v>
       </c>
       <c r="E905" t="s">
-        <v>1121</v>
+        <v>1122</v>
       </c>
       <c r="F905" t="s">
-        <v>1123</v>
+        <v>1133</v>
       </c>
       <c r="G905" t="s">
         <v>1360</v>
@@ -26055,46 +26052,46 @@
         <v>550</v>
       </c>
       <c r="B906" t="s">
-        <v>568</v>
+        <v>569</v>
       </c>
       <c r="C906" t="s">
         <v>1104</v>
       </c>
       <c r="D906">
-        <f>8760 * 0.7 / (7200 * 1000000)</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E906" t="s">
-        <v>1122</v>
+        <v>1130</v>
       </c>
       <c r="F906" t="s">
-        <v>1133</v>
+        <v>1130</v>
       </c>
       <c r="G906" t="s">
-        <v>1361</v>
+        <v>1137</v>
       </c>
     </row>
     <row r="907" spans="1:7">
       <c r="A907" t="s">
-        <v>550</v>
+        <v>551</v>
       </c>
       <c r="B907" t="s">
-        <v>569</v>
+        <v>568</v>
       </c>
       <c r="C907" t="s">
-        <v>1104</v>
+        <v>1105</v>
       </c>
       <c r="D907">
-        <v>1</v>
+        <f>8760 * 0.7 / (7200 * 1000000)</f>
+        <v>0</v>
       </c>
       <c r="E907" t="s">
-        <v>1130</v>
+        <v>1122</v>
       </c>
       <c r="F907" t="s">
-        <v>1130</v>
+        <v>1133</v>
       </c>
       <c r="G907" t="s">
-        <v>1137</v>
+        <v>1360</v>
       </c>
     </row>
     <row r="908" spans="1:7">
@@ -26102,46 +26099,46 @@
         <v>551</v>
       </c>
       <c r="B908" t="s">
-        <v>568</v>
+        <v>569</v>
       </c>
       <c r="C908" t="s">
         <v>1105</v>
       </c>
       <c r="D908">
-        <f>8760 * 0.7 / (7200 * 1000000)</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E908" t="s">
-        <v>1122</v>
+        <v>1130</v>
       </c>
       <c r="F908" t="s">
-        <v>1133</v>
+        <v>1130</v>
       </c>
       <c r="G908" t="s">
-        <v>1361</v>
+        <v>1137</v>
       </c>
     </row>
     <row r="909" spans="1:7">
       <c r="A909" t="s">
-        <v>551</v>
+        <v>552</v>
       </c>
       <c r="B909" t="s">
-        <v>569</v>
+        <v>568</v>
       </c>
       <c r="C909" t="s">
-        <v>1105</v>
+        <v>1106</v>
       </c>
       <c r="D909">
-        <v>1</v>
+        <f>8760 * 0.48 / (4100 * 1000000)</f>
+        <v>0</v>
       </c>
       <c r="E909" t="s">
-        <v>1130</v>
+        <v>1122</v>
       </c>
       <c r="F909" t="s">
-        <v>1130</v>
+        <v>1133</v>
       </c>
       <c r="G909" t="s">
-        <v>1137</v>
+        <v>1361</v>
       </c>
     </row>
     <row r="910" spans="1:7">
@@ -26149,46 +26146,46 @@
         <v>552</v>
       </c>
       <c r="B910" t="s">
-        <v>568</v>
+        <v>569</v>
       </c>
       <c r="C910" t="s">
         <v>1106</v>
       </c>
       <c r="D910">
-        <f>8760 * 0.48 / (4100 * 1000000)</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E910" t="s">
-        <v>1122</v>
+        <v>1130</v>
       </c>
       <c r="F910" t="s">
-        <v>1133</v>
+        <v>1130</v>
       </c>
       <c r="G910" t="s">
-        <v>1362</v>
+        <v>1137</v>
       </c>
     </row>
     <row r="911" spans="1:7">
       <c r="A911" t="s">
-        <v>552</v>
+        <v>553</v>
       </c>
       <c r="B911" t="s">
-        <v>569</v>
+        <v>568</v>
       </c>
       <c r="C911" t="s">
-        <v>1106</v>
+        <v>1107</v>
       </c>
       <c r="D911">
-        <v>1</v>
+        <f>8760 * 0.48 / (4100 * 1000000)</f>
+        <v>0</v>
       </c>
       <c r="E911" t="s">
-        <v>1130</v>
+        <v>1122</v>
       </c>
       <c r="F911" t="s">
-        <v>1130</v>
+        <v>1133</v>
       </c>
       <c r="G911" t="s">
-        <v>1137</v>
+        <v>1361</v>
       </c>
     </row>
     <row r="912" spans="1:7">
@@ -26196,46 +26193,46 @@
         <v>553</v>
       </c>
       <c r="B912" t="s">
-        <v>568</v>
+        <v>569</v>
       </c>
       <c r="C912" t="s">
         <v>1107</v>
       </c>
       <c r="D912">
-        <f>8760 * 0.48 / (4100 * 1000000)</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E912" t="s">
-        <v>1122</v>
+        <v>1130</v>
       </c>
       <c r="F912" t="s">
-        <v>1133</v>
+        <v>1130</v>
       </c>
       <c r="G912" t="s">
-        <v>1362</v>
+        <v>1137</v>
       </c>
     </row>
     <row r="913" spans="1:7">
       <c r="A913" t="s">
-        <v>553</v>
+        <v>554</v>
       </c>
       <c r="B913" t="s">
-        <v>569</v>
+        <v>568</v>
       </c>
       <c r="C913" t="s">
-        <v>1107</v>
+        <v>1108</v>
       </c>
       <c r="D913">
-        <v>1</v>
+        <f>8760 * 0.53 / (5100 * 1000000)</f>
+        <v>0</v>
       </c>
       <c r="E913" t="s">
-        <v>1130</v>
+        <v>1122</v>
       </c>
       <c r="F913" t="s">
-        <v>1130</v>
+        <v>1133</v>
       </c>
       <c r="G913" t="s">
-        <v>1137</v>
+        <v>1362</v>
       </c>
     </row>
     <row r="914" spans="1:7">
@@ -26243,46 +26240,46 @@
         <v>554</v>
       </c>
       <c r="B914" t="s">
-        <v>568</v>
+        <v>569</v>
       </c>
       <c r="C914" t="s">
         <v>1108</v>
       </c>
       <c r="D914">
-        <f>8760 * 0.53 / (5100 * 1000000)</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E914" t="s">
-        <v>1122</v>
+        <v>1130</v>
       </c>
       <c r="F914" t="s">
-        <v>1133</v>
+        <v>1130</v>
       </c>
       <c r="G914" t="s">
-        <v>1363</v>
+        <v>1137</v>
       </c>
     </row>
     <row r="915" spans="1:7">
       <c r="A915" t="s">
-        <v>554</v>
+        <v>555</v>
       </c>
       <c r="B915" t="s">
-        <v>569</v>
+        <v>568</v>
       </c>
       <c r="C915" t="s">
-        <v>1108</v>
+        <v>1109</v>
       </c>
       <c r="D915">
-        <v>1</v>
+        <f>8760 * 0.53 / (5100 * 1000000)</f>
+        <v>0</v>
       </c>
       <c r="E915" t="s">
-        <v>1130</v>
+        <v>1122</v>
       </c>
       <c r="F915" t="s">
-        <v>1130</v>
+        <v>1133</v>
       </c>
       <c r="G915" t="s">
-        <v>1137</v>
+        <v>1362</v>
       </c>
     </row>
     <row r="916" spans="1:7">
@@ -26290,46 +26287,46 @@
         <v>555</v>
       </c>
       <c r="B916" t="s">
-        <v>568</v>
+        <v>569</v>
       </c>
       <c r="C916" t="s">
         <v>1109</v>
       </c>
       <c r="D916">
-        <f>8760 * 0.53 / (5100 * 1000000)</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E916" t="s">
-        <v>1122</v>
+        <v>1130</v>
       </c>
       <c r="F916" t="s">
-        <v>1133</v>
+        <v>1130</v>
       </c>
       <c r="G916" t="s">
-        <v>1363</v>
+        <v>1137</v>
       </c>
     </row>
     <row r="917" spans="1:7">
       <c r="A917" t="s">
-        <v>555</v>
+        <v>556</v>
       </c>
       <c r="B917" t="s">
-        <v>569</v>
+        <v>568</v>
       </c>
       <c r="C917" t="s">
-        <v>1109</v>
+        <v>1110</v>
       </c>
       <c r="D917">
-        <v>1</v>
+        <f>8760 * 0.7 / (7200 * 1000000)</f>
+        <v>0</v>
       </c>
       <c r="E917" t="s">
-        <v>1130</v>
+        <v>1122</v>
       </c>
       <c r="F917" t="s">
-        <v>1130</v>
+        <v>1133</v>
       </c>
       <c r="G917" t="s">
-        <v>1137</v>
+        <v>1360</v>
       </c>
     </row>
     <row r="918" spans="1:7">
@@ -26337,46 +26334,46 @@
         <v>556</v>
       </c>
       <c r="B918" t="s">
-        <v>568</v>
+        <v>569</v>
       </c>
       <c r="C918" t="s">
         <v>1110</v>
       </c>
       <c r="D918">
-        <f>8760 * 0.7 / (7200 * 1000000)</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E918" t="s">
-        <v>1122</v>
+        <v>1130</v>
       </c>
       <c r="F918" t="s">
-        <v>1133</v>
+        <v>1130</v>
       </c>
       <c r="G918" t="s">
-        <v>1361</v>
+        <v>1137</v>
       </c>
     </row>
     <row r="919" spans="1:7">
       <c r="A919" t="s">
-        <v>556</v>
+        <v>557</v>
       </c>
       <c r="B919" t="s">
-        <v>569</v>
+        <v>568</v>
       </c>
       <c r="C919" t="s">
-        <v>1110</v>
+        <v>1111</v>
       </c>
       <c r="D919">
-        <v>1</v>
+        <f>8760 * 0.7 / (7200 * 1000000)</f>
+        <v>0</v>
       </c>
       <c r="E919" t="s">
-        <v>1130</v>
+        <v>1122</v>
       </c>
       <c r="F919" t="s">
-        <v>1130</v>
+        <v>1133</v>
       </c>
       <c r="G919" t="s">
-        <v>1137</v>
+        <v>1360</v>
       </c>
     </row>
     <row r="920" spans="1:7">
@@ -26384,46 +26381,46 @@
         <v>557</v>
       </c>
       <c r="B920" t="s">
-        <v>568</v>
+        <v>569</v>
       </c>
       <c r="C920" t="s">
         <v>1111</v>
       </c>
       <c r="D920">
-        <f>8760 * 0.7 / (7200 * 1000000)</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E920" t="s">
-        <v>1122</v>
+        <v>1130</v>
       </c>
       <c r="F920" t="s">
-        <v>1133</v>
+        <v>1130</v>
       </c>
       <c r="G920" t="s">
-        <v>1361</v>
+        <v>1137</v>
       </c>
     </row>
     <row r="921" spans="1:7">
       <c r="A921" t="s">
-        <v>557</v>
+        <v>558</v>
       </c>
       <c r="B921" t="s">
-        <v>569</v>
+        <v>568</v>
       </c>
       <c r="C921" t="s">
-        <v>1111</v>
+        <v>1112</v>
       </c>
       <c r="D921">
-        <v>1</v>
+        <f>8760 * 0.48 / (4100 * 1000000)</f>
+        <v>0</v>
       </c>
       <c r="E921" t="s">
-        <v>1130</v>
+        <v>1122</v>
       </c>
       <c r="F921" t="s">
-        <v>1130</v>
+        <v>1133</v>
       </c>
       <c r="G921" t="s">
-        <v>1137</v>
+        <v>1361</v>
       </c>
     </row>
     <row r="922" spans="1:7">
@@ -26431,46 +26428,46 @@
         <v>558</v>
       </c>
       <c r="B922" t="s">
-        <v>568</v>
+        <v>569</v>
       </c>
       <c r="C922" t="s">
         <v>1112</v>
       </c>
       <c r="D922">
-        <f>8760 * 0.48 / (4100 * 1000000)</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E922" t="s">
-        <v>1122</v>
+        <v>1130</v>
       </c>
       <c r="F922" t="s">
-        <v>1133</v>
+        <v>1130</v>
       </c>
       <c r="G922" t="s">
-        <v>1362</v>
+        <v>1137</v>
       </c>
     </row>
     <row r="923" spans="1:7">
       <c r="A923" t="s">
-        <v>558</v>
+        <v>559</v>
       </c>
       <c r="B923" t="s">
-        <v>569</v>
+        <v>568</v>
       </c>
       <c r="C923" t="s">
-        <v>1112</v>
+        <v>1113</v>
       </c>
       <c r="D923">
-        <v>1</v>
+        <f>8760 * 0.48 / (4100 * 1000000)</f>
+        <v>0</v>
       </c>
       <c r="E923" t="s">
-        <v>1130</v>
+        <v>1122</v>
       </c>
       <c r="F923" t="s">
-        <v>1130</v>
+        <v>1133</v>
       </c>
       <c r="G923" t="s">
-        <v>1137</v>
+        <v>1361</v>
       </c>
     </row>
     <row r="924" spans="1:7">
@@ -26478,46 +26475,46 @@
         <v>559</v>
       </c>
       <c r="B924" t="s">
-        <v>568</v>
+        <v>569</v>
       </c>
       <c r="C924" t="s">
         <v>1113</v>
       </c>
       <c r="D924">
-        <f>8760 * 0.48 / (4100 * 1000000)</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E924" t="s">
-        <v>1122</v>
+        <v>1130</v>
       </c>
       <c r="F924" t="s">
-        <v>1133</v>
+        <v>1130</v>
       </c>
       <c r="G924" t="s">
-        <v>1362</v>
+        <v>1137</v>
       </c>
     </row>
     <row r="925" spans="1:7">
       <c r="A925" t="s">
-        <v>559</v>
+        <v>560</v>
       </c>
       <c r="B925" t="s">
-        <v>569</v>
+        <v>568</v>
       </c>
       <c r="C925" t="s">
-        <v>1113</v>
+        <v>1114</v>
       </c>
       <c r="D925">
-        <v>1</v>
+        <f>8760 * 0.53 / (5100 * 1000000)</f>
+        <v>0</v>
       </c>
       <c r="E925" t="s">
-        <v>1130</v>
+        <v>1122</v>
       </c>
       <c r="F925" t="s">
-        <v>1130</v>
+        <v>1133</v>
       </c>
       <c r="G925" t="s">
-        <v>1137</v>
+        <v>1362</v>
       </c>
     </row>
     <row r="926" spans="1:7">
@@ -26525,46 +26522,46 @@
         <v>560</v>
       </c>
       <c r="B926" t="s">
-        <v>568</v>
+        <v>569</v>
       </c>
       <c r="C926" t="s">
         <v>1114</v>
       </c>
       <c r="D926">
-        <f>8760 * 0.53 / (5100 * 1000000)</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E926" t="s">
-        <v>1122</v>
+        <v>1130</v>
       </c>
       <c r="F926" t="s">
-        <v>1133</v>
+        <v>1130</v>
       </c>
       <c r="G926" t="s">
-        <v>1363</v>
+        <v>1137</v>
       </c>
     </row>
     <row r="927" spans="1:7">
       <c r="A927" t="s">
-        <v>560</v>
+        <v>561</v>
       </c>
       <c r="B927" t="s">
-        <v>569</v>
+        <v>568</v>
       </c>
       <c r="C927" t="s">
-        <v>1114</v>
+        <v>1115</v>
       </c>
       <c r="D927">
-        <v>1</v>
+        <f>8760 * 0.53 / (5100 * 1000000)</f>
+        <v>0</v>
       </c>
       <c r="E927" t="s">
-        <v>1130</v>
+        <v>1122</v>
       </c>
       <c r="F927" t="s">
-        <v>1130</v>
+        <v>1133</v>
       </c>
       <c r="G927" t="s">
-        <v>1137</v>
+        <v>1362</v>
       </c>
     </row>
     <row r="928" spans="1:7">
@@ -26572,43 +26569,42 @@
         <v>561</v>
       </c>
       <c r="B928" t="s">
-        <v>568</v>
+        <v>569</v>
       </c>
       <c r="C928" t="s">
         <v>1115</v>
       </c>
       <c r="D928">
-        <f>8760 * 0.53 / (5100 * 1000000)</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E928" t="s">
-        <v>1122</v>
+        <v>1130</v>
       </c>
       <c r="F928" t="s">
-        <v>1133</v>
+        <v>1130</v>
       </c>
       <c r="G928" t="s">
-        <v>1363</v>
+        <v>1137</v>
       </c>
     </row>
     <row r="929" spans="1:7">
       <c r="A929" t="s">
-        <v>561</v>
+        <v>562</v>
       </c>
       <c r="B929" t="s">
         <v>569</v>
       </c>
       <c r="C929" t="s">
-        <v>1115</v>
+        <v>1116</v>
       </c>
       <c r="D929">
         <v>1</v>
       </c>
       <c r="E929" t="s">
-        <v>1130</v>
+        <v>1121</v>
       </c>
       <c r="F929" t="s">
-        <v>1130</v>
+        <v>1121</v>
       </c>
       <c r="G929" t="s">
         <v>1137</v>
@@ -26616,13 +26612,13 @@
     </row>
     <row r="930" spans="1:7">
       <c r="A930" t="s">
-        <v>562</v>
+        <v>563</v>
       </c>
       <c r="B930" t="s">
         <v>569</v>
       </c>
       <c r="C930" t="s">
-        <v>1116</v>
+        <v>1117</v>
       </c>
       <c r="D930">
         <v>1</v>
@@ -26639,13 +26635,13 @@
     </row>
     <row r="931" spans="1:7">
       <c r="A931" t="s">
-        <v>563</v>
+        <v>564</v>
       </c>
       <c r="B931" t="s">
         <v>569</v>
       </c>
       <c r="C931" t="s">
-        <v>1117</v>
+        <v>1118</v>
       </c>
       <c r="D931">
         <v>1</v>
@@ -26662,13 +26658,13 @@
     </row>
     <row r="932" spans="1:7">
       <c r="A932" t="s">
-        <v>564</v>
+        <v>565</v>
       </c>
       <c r="B932" t="s">
         <v>569</v>
       </c>
       <c r="C932" t="s">
-        <v>1118</v>
+        <v>1119</v>
       </c>
       <c r="D932">
         <v>1</v>
@@ -26685,13 +26681,13 @@
     </row>
     <row r="933" spans="1:7">
       <c r="A933" t="s">
-        <v>565</v>
+        <v>566</v>
       </c>
       <c r="B933" t="s">
         <v>569</v>
       </c>
       <c r="C933" t="s">
-        <v>1119</v>
+        <v>1120</v>
       </c>
       <c r="D933">
         <v>1</v>
@@ -26703,29 +26699,6 @@
         <v>1121</v>
       </c>
       <c r="G933" t="s">
-        <v>1137</v>
-      </c>
-    </row>
-    <row r="934" spans="1:7">
-      <c r="A934" t="s">
-        <v>566</v>
-      </c>
-      <c r="B934" t="s">
-        <v>569</v>
-      </c>
-      <c r="C934" t="s">
-        <v>1120</v>
-      </c>
-      <c r="D934">
-        <v>1</v>
-      </c>
-      <c r="E934" t="s">
-        <v>1121</v>
-      </c>
-      <c r="F934" t="s">
-        <v>1121</v>
-      </c>
-      <c r="G934" t="s">
         <v>1137</v>
       </c>
     </row>

</xml_diff>